<commit_message>
added the marker to the billboards
</commit_message>
<xml_diff>
--- a/_trackers/Ticker_Company_Names.xlsx
+++ b/_trackers/Ticker_Company_Names.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sugit\Documents\Claude\_Stock_agent\_trackers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F000B9CC-B4D5-41B1-B426-614D961B5D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BEE9798-245A-474D-964D-F31D6EC509E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1081,13 +1081,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1498,7 +1497,7 @@
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="4"/>
+      <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -1507,7 +1506,7 @@
       <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="9" t="s">
         <v>301</v>
       </c>
     </row>
@@ -1518,18 +1517,18 @@
       <c r="B4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="13" t="s">
         <v>302</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="8" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="9" t="s">
         <v>303</v>
       </c>
     </row>
@@ -1540,69 +1539,69 @@
       <c r="B6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="9" t="s">
         <v>304</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="8" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="9" t="s">
         <v>305</v>
       </c>
-      <c r="E7" s="4"/>
+      <c r="E7" s="3"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>14</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="9" t="s">
         <v>306</v>
       </c>
-      <c r="E8" s="4"/>
+      <c r="E8" s="3"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="8" t="s">
         <v>16</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="12" t="s">
         <v>307</v>
       </c>
-      <c r="E9" s="4"/>
+      <c r="E9" s="3"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="8" t="s">
         <v>18</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="10" t="s">
         <v>308</v>
       </c>
-      <c r="E10" s="4"/>
+      <c r="E10" s="3"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="14" t="s">
         <v>20</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="E11" s="4"/>
+      <c r="E11" s="3"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
@@ -1611,10 +1610,10 @@
       <c r="B12" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="11" t="s">
         <v>310</v>
       </c>
-      <c r="E12" s="4"/>
+      <c r="E12" s="3"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
@@ -1623,30 +1622,30 @@
       <c r="B13" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="13" t="s">
         <v>311</v>
       </c>
-      <c r="E13" s="4"/>
+      <c r="E13" s="3"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="8" t="s">
         <v>26</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="D14" s="13" t="s">
         <v>312</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="8" t="s">
         <v>28</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="9" t="s">
         <v>313</v>
       </c>
     </row>
@@ -1657,21 +1656,21 @@
       <c r="B16" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="D16" s="13" t="s">
         <v>314</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="8" t="s">
         <v>32</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="D17" s="13" t="s">
         <v>315</v>
       </c>
-      <c r="E17" s="4"/>
+      <c r="E17" s="3"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
@@ -1680,31 +1679,31 @@
       <c r="B18" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="8" t="s">
         <v>36</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
+      <c r="A20" s="14" t="s">
         <v>38</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="15" t="s">
+      <c r="A21" s="14" t="s">
         <v>40</v>
       </c>
       <c r="B21" s="2" t="s">
@@ -1712,17 +1711,17 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="14" t="s">
         <v>42</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="14" t="s">
         <v>44</v>
       </c>
       <c r="B23" s="2" t="s">
@@ -1736,8 +1735,8 @@
       <c r="B24" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
@@ -1754,7 +1753,7 @@
       <c r="B26" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D26" s="4"/>
+      <c r="D26" s="3"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
@@ -1771,7 +1770,7 @@
       <c r="B28" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D28" s="4"/>
+      <c r="D28" s="3"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
@@ -1788,7 +1787,7 @@
       <c r="B30" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D30" s="4"/>
+      <c r="D30" s="3"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
@@ -1805,7 +1804,7 @@
       <c r="B32" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D32" s="4"/>
+      <c r="D32" s="3"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
@@ -1814,7 +1813,7 @@
       <c r="B33" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D33" s="4"/>
+      <c r="D33" s="3"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
@@ -1823,7 +1822,7 @@
       <c r="B34" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D34" s="4"/>
+      <c r="D34" s="3"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
@@ -1832,7 +1831,7 @@
       <c r="B35" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D35" s="4"/>
+      <c r="D35" s="3"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
@@ -2025,7 +2024,7 @@
       <c r="B59" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="E59" s="4"/>
+      <c r="E59" s="3"/>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
@@ -2034,7 +2033,7 @@
       <c r="B60" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="E60" s="4"/>
+      <c r="E60" s="3"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
@@ -2043,7 +2042,7 @@
       <c r="B61" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="E61" s="4"/>
+      <c r="E61" s="3"/>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
@@ -2052,7 +2051,7 @@
       <c r="B62" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="E62" s="4"/>
+      <c r="E62" s="3"/>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
@@ -2061,7 +2060,7 @@
       <c r="B63" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="E63" s="4"/>
+      <c r="E63" s="3"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
@@ -2070,7 +2069,7 @@
       <c r="B64" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="E64" s="4"/>
+      <c r="E64" s="3"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
@@ -2079,7 +2078,7 @@
       <c r="B65" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="E65" s="4"/>
+      <c r="E65" s="3"/>
     </row>
     <row r="66" spans="1:5" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
@@ -2088,7 +2087,7 @@
       <c r="B66" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="E66" s="5"/>
+      <c r="E66" s="4"/>
     </row>
     <row r="67" spans="1:5" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
@@ -2097,7 +2096,7 @@
       <c r="B67" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E67" s="6"/>
+      <c r="E67" s="5"/>
     </row>
     <row r="68" spans="1:5" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
@@ -2106,7 +2105,7 @@
       <c r="B68" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="E68" s="6"/>
+      <c r="E68" s="5"/>
     </row>
     <row r="69" spans="1:5" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
@@ -2115,7 +2114,7 @@
       <c r="B69" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="E69" s="6"/>
+      <c r="E69" s="5"/>
     </row>
     <row r="70" spans="1:5" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
@@ -2124,7 +2123,7 @@
       <c r="B70" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="E70" s="5"/>
+      <c r="E70" s="4"/>
     </row>
     <row r="71" spans="1:5" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
@@ -2133,7 +2132,7 @@
       <c r="B71" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="E71" s="6"/>
+      <c r="E71" s="5"/>
     </row>
     <row r="72" spans="1:5" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
@@ -2142,7 +2141,7 @@
       <c r="B72" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="E72" s="5"/>
+      <c r="E72" s="4"/>
     </row>
     <row r="73" spans="1:5" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
@@ -2151,7 +2150,7 @@
       <c r="B73" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="E73" s="7"/>
+      <c r="E73" s="6"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
@@ -2160,7 +2159,7 @@
       <c r="B74" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="E74" s="8"/>
+      <c r="E74" s="7"/>
     </row>
     <row r="75" spans="1:5" ht="20.399999999999999" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
@@ -2169,7 +2168,7 @@
       <c r="B75" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E75" s="7"/>
+      <c r="E75" s="6"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">

</xml_diff>